<commit_message>
bouton stop intégré à l'ui
</commit_message>
<xml_diff>
--- a/Suivi_Comportemental_Challenger.xlsx
+++ b/Suivi_Comportemental_Challenger.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2599" uniqueCount="573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2690" uniqueCount="583">
   <si>
     <t>Date</t>
   </si>
@@ -1264,6 +1264,36 @@
     <t>42:56</t>
   </si>
   <si>
+    <t>35:22</t>
+  </si>
+  <si>
+    <t>18:14</t>
+  </si>
+  <si>
+    <t>23:21</t>
+  </si>
+  <si>
+    <t>1:11</t>
+  </si>
+  <si>
+    <t>24/03/2026</t>
+  </si>
+  <si>
+    <t>22:23</t>
+  </si>
+  <si>
+    <t>23:01</t>
+  </si>
+  <si>
+    <t>29:06</t>
+  </si>
+  <si>
+    <t>21:10</t>
+  </si>
+  <si>
+    <t>34:22</t>
+  </si>
+  <si>
     <t>Stats par Champion  —  trie par parties jouees</t>
   </si>
   <si>
@@ -1312,6 +1342,9 @@
     <t>Duree Moy.</t>
   </si>
   <si>
+    <t>28:15</t>
+  </si>
+  <si>
     <t>28:57</t>
   </si>
   <si>
@@ -1321,18 +1354,18 @@
     <t>30:34</t>
   </si>
   <si>
-    <t>29:51</t>
-  </si>
-  <si>
-    <t>25:55</t>
+    <t>26:43</t>
+  </si>
+  <si>
+    <t>25:45</t>
+  </si>
+  <si>
+    <t>31:50</t>
   </si>
   <si>
     <t>23:27</t>
   </si>
   <si>
-    <t>32:44</t>
-  </si>
-  <si>
     <t>Comparaison Solo vs Duo</t>
   </si>
   <si>
@@ -1408,19 +1441,19 @@
     <t>KDA moyen</t>
   </si>
   <si>
-    <t>3.40</t>
+    <t>3.38</t>
   </si>
   <si>
     <t>K / D / A moyens</t>
   </si>
   <si>
-    <t>10.8 / 8.0 / 6.8</t>
+    <t>10.7 / 7.9 / 6.8</t>
   </si>
   <si>
     <t>CS/Min moyen</t>
   </si>
   <si>
-    <t>6.8</t>
+    <t>6.7</t>
   </si>
   <si>
     <t>DPM moyen</t>
@@ -1432,19 +1465,19 @@
     <t>% DMG Equipe moyen</t>
   </si>
   <si>
-    <t>27.7 %</t>
+    <t>28.3 %</t>
   </si>
   <si>
     <t>KP % moyen</t>
   </si>
   <si>
-    <t>54.2 %</t>
+    <t>54.0 %</t>
   </si>
   <si>
     <t>Vision Score moyen</t>
   </si>
   <si>
-    <t>23.1</t>
+    <t>22.9</t>
   </si>
   <si>
     <t>Serie Actuelle &amp; Tendance</t>
@@ -1498,73 +1531,73 @@
     <t>Partie 1</t>
   </si>
   <si>
-    <t>3.63</t>
-  </si>
-  <si>
-    <t>12.4</t>
-  </si>
-  <si>
-    <t>7.8</t>
-  </si>
-  <si>
-    <t>6.0</t>
-  </si>
-  <si>
-    <t>6.7 | 1069</t>
+    <t>3.67</t>
+  </si>
+  <si>
+    <t>12.3</t>
+  </si>
+  <si>
+    <t>7.5</t>
+  </si>
+  <si>
+    <t>5.9</t>
+  </si>
+  <si>
+    <t>6.6 | 1105</t>
   </si>
   <si>
     <t>Partie 2</t>
   </si>
   <si>
-    <t>4.07</t>
-  </si>
-  <si>
-    <t>7.2</t>
-  </si>
-  <si>
-    <t>8.4</t>
-  </si>
-  <si>
-    <t>7.7 | 1186</t>
+    <t>3.92</t>
+  </si>
+  <si>
+    <t>12.1</t>
+  </si>
+  <si>
+    <t>7.0</t>
+  </si>
+  <si>
+    <t>7.4</t>
+  </si>
+  <si>
+    <t>7.6 | 1171</t>
   </si>
   <si>
     <t>Partie 3</t>
   </si>
   <si>
-    <t>4.71</t>
-  </si>
-  <si>
-    <t>13.7</t>
-  </si>
-  <si>
-    <t>7.6</t>
-  </si>
-  <si>
-    <t>7.3</t>
-  </si>
-  <si>
-    <t>7.6 | 1314</t>
+    <t>3.87</t>
+  </si>
+  <si>
+    <t>13.4</t>
+  </si>
+  <si>
+    <t>8.0</t>
+  </si>
+  <si>
+    <t>7.5 | 1284</t>
   </si>
   <si>
     <t>Partie 4+</t>
   </si>
   <si>
-    <t>2.80</t>
-  </si>
-  <si>
-    <t>9.2</t>
-  </si>
-  <si>
-    <t>8.3</t>
-  </si>
-  <si>
-    <t>6.4</t>
-  </si>
-  <si>
-    <t>6.3 | 982</t>
-  </si>
-  <si>
-    <t>Diagnostic : ⚠ Fatigue forte (-19.3% WR P1→P4+)</t>
+    <t>3.02</t>
+  </si>
+  <si>
+    <t>9.1</t>
+  </si>
+  <si>
+    <t>8.2</t>
+  </si>
+  <si>
+    <t>6.6</t>
+  </si>
+  <si>
+    <t>6.4 | 982</t>
+  </si>
+  <si>
+    <t>Diagnostic : ! Legere fatigue (-14.8% WR P1→P4+)</t>
   </si>
   <si>
     <t>Performance par Tranche Horaire</t>
@@ -1609,10 +1642,10 @@
     <t>Soir (18h-24h)</t>
   </si>
   <si>
-    <t>3.18</t>
-  </si>
-  <si>
-    <t>10.4/8.1/6.5</t>
+    <t>3.17</t>
+  </si>
+  <si>
+    <t>10.2/8.0/6.5</t>
   </si>
   <si>
     <t>Neutre</t>
@@ -1627,10 +1660,10 @@
     <t>Apres une Victoire</t>
   </si>
   <si>
-    <t>4.24</t>
-  </si>
-  <si>
-    <t>11.4/7.2/7.0</t>
+    <t>4.17</t>
+  </si>
+  <si>
+    <t>11.2/7.1/6.9</t>
   </si>
   <si>
     <t/>
@@ -1639,10 +1672,10 @@
     <t>Apres une Defaite</t>
   </si>
   <si>
-    <t>2.54</t>
-  </si>
-  <si>
-    <t>10.3/8.7/6.5</t>
+    <t>2.52</t>
+  </si>
+  <si>
+    <t>10.1/8.7/6.6</t>
   </si>
   <si>
     <t>Tilt detecte — Stopper apres defaite</t>
@@ -1669,10 +1702,10 @@
     <t>0 gank(s) mortel(s)</t>
   </si>
   <si>
-    <t>4.88</t>
-  </si>
-  <si>
-    <t>10.2/6.3/6.2</t>
+    <t>4.75</t>
+  </si>
+  <si>
+    <t>9.8/6.2/6.1</t>
   </si>
   <si>
     <t>Excellente resistance</t>
@@ -1681,10 +1714,7 @@
     <t>1 gank(s) mortel(s)</t>
   </si>
   <si>
-    <t>3.20</t>
-  </si>
-  <si>
-    <t>11.3/8.3/6.7</t>
+    <t>11.3/8.4/6.8</t>
   </si>
   <si>
     <t>Stable</t>
@@ -1693,19 +1723,19 @@
     <t>2 gank(s) mortel(s)</t>
   </si>
   <si>
-    <t>2.64</t>
-  </si>
-  <si>
-    <t>12.6/8.5/7.9</t>
+    <t>2.83</t>
+  </si>
+  <si>
+    <t>12.7/8.3/8.0</t>
   </si>
   <si>
     <t>3+ ganks mortels</t>
   </si>
   <si>
-    <t>1.62</t>
-  </si>
-  <si>
-    <t>8.3/9.8/6.4</t>
+    <t>1.57</t>
+  </si>
+  <si>
+    <t>8.0/9.8/6.3</t>
   </si>
   <si>
     <t>Impact critique</t>
@@ -2484,7 +2514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BB151"/>
+  <dimension ref="A1:BB157"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2693,7 +2723,7 @@
         <v>55</v>
       </c>
       <c r="C2" s="10">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2" s="10">
         <v>3</v>
@@ -2857,7 +2887,7 @@
         <v>67</v>
       </c>
       <c r="C3" s="24">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" s="24">
         <v>2</v>
@@ -3021,7 +3051,7 @@
         <v>72</v>
       </c>
       <c r="C4" s="10">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" s="10">
         <v>1</v>
@@ -3185,7 +3215,7 @@
         <v>78</v>
       </c>
       <c r="C5" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D5" s="24">
         <v>8</v>
@@ -3349,7 +3379,7 @@
         <v>85</v>
       </c>
       <c r="C6" s="10">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="10">
         <v>7</v>
@@ -3513,7 +3543,7 @@
         <v>90</v>
       </c>
       <c r="C7" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D7" s="24">
         <v>6</v>
@@ -3677,7 +3707,7 @@
         <v>93</v>
       </c>
       <c r="C8" s="10">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" s="10">
         <v>5</v>
@@ -3841,7 +3871,7 @@
         <v>96</v>
       </c>
       <c r="C9" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="24">
         <v>4</v>
@@ -4005,7 +4035,7 @@
         <v>100</v>
       </c>
       <c r="C10" s="10">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D10" s="10">
         <v>3</v>
@@ -4169,7 +4199,7 @@
         <v>103</v>
       </c>
       <c r="C11" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D11" s="24">
         <v>2</v>
@@ -4333,7 +4363,7 @@
         <v>106</v>
       </c>
       <c r="C12" s="10">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D12" s="10">
         <v>1</v>
@@ -4497,7 +4527,7 @@
         <v>109</v>
       </c>
       <c r="C13" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="24">
         <v>9</v>
@@ -4661,7 +4691,7 @@
         <v>112</v>
       </c>
       <c r="C14" s="10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" s="10">
         <v>8</v>
@@ -4825,7 +4855,7 @@
         <v>55</v>
       </c>
       <c r="C15" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15" s="24">
         <v>7</v>
@@ -4989,7 +5019,7 @@
         <v>116</v>
       </c>
       <c r="C16" s="10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="10">
         <v>6</v>
@@ -5153,7 +5183,7 @@
         <v>119</v>
       </c>
       <c r="C17" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="24">
         <v>5</v>
@@ -5317,7 +5347,7 @@
         <v>122</v>
       </c>
       <c r="C18" s="10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D18" s="10">
         <v>4</v>
@@ -5481,7 +5511,7 @@
         <v>124</v>
       </c>
       <c r="C19" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D19" s="24">
         <v>3</v>
@@ -5645,7 +5675,7 @@
         <v>126</v>
       </c>
       <c r="C20" s="10">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D20" s="10">
         <v>2</v>
@@ -5809,7 +5839,7 @@
         <v>128</v>
       </c>
       <c r="C21" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D21" s="24">
         <v>1</v>
@@ -5973,7 +6003,7 @@
         <v>130</v>
       </c>
       <c r="C22" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D22" s="10">
         <v>7</v>
@@ -6137,7 +6167,7 @@
         <v>133</v>
       </c>
       <c r="C23" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D23" s="24">
         <v>6</v>
@@ -6301,7 +6331,7 @@
         <v>135</v>
       </c>
       <c r="C24" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D24" s="10">
         <v>5</v>
@@ -6465,7 +6495,7 @@
         <v>139</v>
       </c>
       <c r="C25" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D25" s="24">
         <v>4</v>
@@ -6629,7 +6659,7 @@
         <v>141</v>
       </c>
       <c r="C26" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D26" s="10">
         <v>3</v>
@@ -6793,7 +6823,7 @@
         <v>144</v>
       </c>
       <c r="C27" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D27" s="24">
         <v>2</v>
@@ -6957,7 +6987,7 @@
         <v>146</v>
       </c>
       <c r="C28" s="10">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D28" s="10">
         <v>1</v>
@@ -7121,7 +7151,7 @@
         <v>149</v>
       </c>
       <c r="C29" s="24">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D29" s="24">
         <v>4</v>
@@ -7285,7 +7315,7 @@
         <v>151</v>
       </c>
       <c r="C30" s="10">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D30" s="10">
         <v>3</v>
@@ -7449,7 +7479,7 @@
         <v>154</v>
       </c>
       <c r="C31" s="24">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D31" s="24">
         <v>2</v>
@@ -7613,7 +7643,7 @@
         <v>156</v>
       </c>
       <c r="C32" s="10">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D32" s="10">
         <v>1</v>
@@ -7777,7 +7807,7 @@
         <v>158</v>
       </c>
       <c r="C33" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D33" s="24">
         <v>9</v>
@@ -7941,7 +7971,7 @@
         <v>160</v>
       </c>
       <c r="C34" s="10">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D34" s="10">
         <v>8</v>
@@ -8105,7 +8135,7 @@
         <v>164</v>
       </c>
       <c r="C35" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D35" s="24">
         <v>7</v>
@@ -8269,7 +8299,7 @@
         <v>167</v>
       </c>
       <c r="C36" s="10">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D36" s="10">
         <v>6</v>
@@ -8433,7 +8463,7 @@
         <v>170</v>
       </c>
       <c r="C37" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D37" s="24">
         <v>5</v>
@@ -8597,7 +8627,7 @@
         <v>85</v>
       </c>
       <c r="C38" s="10">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D38" s="10">
         <v>4</v>
@@ -8761,7 +8791,7 @@
         <v>174</v>
       </c>
       <c r="C39" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D39" s="24">
         <v>3</v>
@@ -8925,7 +8955,7 @@
         <v>176</v>
       </c>
       <c r="C40" s="10">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D40" s="10">
         <v>2</v>
@@ -9089,7 +9119,7 @@
         <v>178</v>
       </c>
       <c r="C41" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D41" s="24">
         <v>1</v>
@@ -9253,7 +9283,7 @@
         <v>180</v>
       </c>
       <c r="C42" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D42" s="10">
         <v>9</v>
@@ -9417,7 +9447,7 @@
         <v>183</v>
       </c>
       <c r="C43" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D43" s="24">
         <v>8</v>
@@ -9581,7 +9611,7 @@
         <v>186</v>
       </c>
       <c r="C44" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D44" s="10">
         <v>7</v>
@@ -9745,7 +9775,7 @@
         <v>189</v>
       </c>
       <c r="C45" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D45" s="24">
         <v>6</v>
@@ -9909,7 +9939,7 @@
         <v>192</v>
       </c>
       <c r="C46" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D46" s="10">
         <v>5</v>
@@ -10073,7 +10103,7 @@
         <v>194</v>
       </c>
       <c r="C47" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D47" s="24">
         <v>4</v>
@@ -10237,7 +10267,7 @@
         <v>197</v>
       </c>
       <c r="C48" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D48" s="10">
         <v>3</v>
@@ -10401,7 +10431,7 @@
         <v>200</v>
       </c>
       <c r="C49" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D49" s="24">
         <v>2</v>
@@ -10565,7 +10595,7 @@
         <v>203</v>
       </c>
       <c r="C50" s="10">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D50" s="10">
         <v>1</v>
@@ -10729,7 +10759,7 @@
         <v>206</v>
       </c>
       <c r="C51" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D51" s="24">
         <v>1</v>
@@ -10893,7 +10923,7 @@
         <v>209</v>
       </c>
       <c r="C52" s="10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D52" s="10">
         <v>6</v>
@@ -11057,7 +11087,7 @@
         <v>212</v>
       </c>
       <c r="C53" s="24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D53" s="24">
         <v>5</v>
@@ -11221,7 +11251,7 @@
         <v>214</v>
       </c>
       <c r="C54" s="10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D54" s="10">
         <v>4</v>
@@ -11385,7 +11415,7 @@
         <v>217</v>
       </c>
       <c r="C55" s="24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D55" s="24">
         <v>3</v>
@@ -11549,7 +11579,7 @@
         <v>219</v>
       </c>
       <c r="C56" s="10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D56" s="10">
         <v>2</v>
@@ -11713,7 +11743,7 @@
         <v>221</v>
       </c>
       <c r="C57" s="24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D57" s="24">
         <v>1</v>
@@ -11877,7 +11907,7 @@
         <v>225</v>
       </c>
       <c r="C58" s="10">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D58" s="10">
         <v>6</v>
@@ -12041,7 +12071,7 @@
         <v>112</v>
       </c>
       <c r="C59" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D59" s="24">
         <v>5</v>
@@ -12205,7 +12235,7 @@
         <v>227</v>
       </c>
       <c r="C60" s="10">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D60" s="10">
         <v>4</v>
@@ -12369,7 +12399,7 @@
         <v>229</v>
       </c>
       <c r="C61" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D61" s="24">
         <v>3</v>
@@ -12533,7 +12563,7 @@
         <v>231</v>
       </c>
       <c r="C62" s="10">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D62" s="10">
         <v>2</v>
@@ -12697,7 +12727,7 @@
         <v>233</v>
       </c>
       <c r="C63" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D63" s="24">
         <v>1</v>
@@ -12861,7 +12891,7 @@
         <v>112</v>
       </c>
       <c r="C64" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D64" s="10">
         <v>6</v>
@@ -13025,7 +13055,7 @@
         <v>194</v>
       </c>
       <c r="C65" s="24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D65" s="24">
         <v>5</v>
@@ -13189,7 +13219,7 @@
         <v>240</v>
       </c>
       <c r="C66" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D66" s="10">
         <v>4</v>
@@ -13353,7 +13383,7 @@
         <v>242</v>
       </c>
       <c r="C67" s="24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D67" s="24">
         <v>3</v>
@@ -13517,7 +13547,7 @@
         <v>244</v>
       </c>
       <c r="C68" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D68" s="10">
         <v>2</v>
@@ -13681,7 +13711,7 @@
         <v>246</v>
       </c>
       <c r="C69" s="24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D69" s="24">
         <v>1</v>
@@ -13845,7 +13875,7 @@
         <v>250</v>
       </c>
       <c r="C70" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D70" s="10">
         <v>9</v>
@@ -14009,7 +14039,7 @@
         <v>253</v>
       </c>
       <c r="C71" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D71" s="24">
         <v>8</v>
@@ -14173,7 +14203,7 @@
         <v>255</v>
       </c>
       <c r="C72" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D72" s="10">
         <v>7</v>
@@ -14337,7 +14367,7 @@
         <v>257</v>
       </c>
       <c r="C73" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D73" s="24">
         <v>6</v>
@@ -14501,7 +14531,7 @@
         <v>260</v>
       </c>
       <c r="C74" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D74" s="10">
         <v>5</v>
@@ -14665,7 +14695,7 @@
         <v>116</v>
       </c>
       <c r="C75" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D75" s="24">
         <v>4</v>
@@ -14829,7 +14859,7 @@
         <v>263</v>
       </c>
       <c r="C76" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D76" s="10">
         <v>3</v>
@@ -14993,7 +15023,7 @@
         <v>144</v>
       </c>
       <c r="C77" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D77" s="24">
         <v>2</v>
@@ -15157,7 +15187,7 @@
         <v>219</v>
       </c>
       <c r="C78" s="10">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D78" s="10">
         <v>1</v>
@@ -15321,7 +15351,7 @@
         <v>267</v>
       </c>
       <c r="C79" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D79" s="24">
         <v>1</v>
@@ -15485,7 +15515,7 @@
         <v>269</v>
       </c>
       <c r="C80" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D80" s="10">
         <v>9</v>
@@ -15649,7 +15679,7 @@
         <v>271</v>
       </c>
       <c r="C81" s="24">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D81" s="24">
         <v>8</v>
@@ -15813,7 +15843,7 @@
         <v>274</v>
       </c>
       <c r="C82" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D82" s="10">
         <v>7</v>
@@ -15977,7 +16007,7 @@
         <v>276</v>
       </c>
       <c r="C83" s="24">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D83" s="24">
         <v>6</v>
@@ -16141,7 +16171,7 @@
         <v>170</v>
       </c>
       <c r="C84" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D84" s="10">
         <v>5</v>
@@ -16305,7 +16335,7 @@
         <v>280</v>
       </c>
       <c r="C85" s="24">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D85" s="24">
         <v>4</v>
@@ -16469,7 +16499,7 @@
         <v>282</v>
       </c>
       <c r="C86" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D86" s="10">
         <v>3</v>
@@ -16633,7 +16663,7 @@
         <v>157</v>
       </c>
       <c r="C87" s="24">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D87" s="24">
         <v>2</v>
@@ -16797,7 +16827,7 @@
         <v>285</v>
       </c>
       <c r="C88" s="10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D88" s="10">
         <v>1</v>
@@ -16961,7 +16991,7 @@
         <v>288</v>
       </c>
       <c r="C89" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D89" s="24">
         <v>9</v>
@@ -17125,7 +17155,7 @@
         <v>290</v>
       </c>
       <c r="C90" s="10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D90" s="10">
         <v>8</v>
@@ -17289,7 +17319,7 @@
         <v>292</v>
       </c>
       <c r="C91" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D91" s="24">
         <v>7</v>
@@ -17453,7 +17483,7 @@
         <v>294</v>
       </c>
       <c r="C92" s="10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D92" s="10">
         <v>6</v>
@@ -17617,7 +17647,7 @@
         <v>93</v>
       </c>
       <c r="C93" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D93" s="24">
         <v>5</v>
@@ -17781,7 +17811,7 @@
         <v>298</v>
       </c>
       <c r="C94" s="10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D94" s="10">
         <v>4</v>
@@ -17945,7 +17975,7 @@
         <v>300</v>
       </c>
       <c r="C95" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D95" s="24">
         <v>3</v>
@@ -18109,7 +18139,7 @@
         <v>302</v>
       </c>
       <c r="C96" s="10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D96" s="10">
         <v>2</v>
@@ -18273,7 +18303,7 @@
         <v>304</v>
       </c>
       <c r="C97" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D97" s="24">
         <v>1</v>
@@ -18437,7 +18467,7 @@
         <v>307</v>
       </c>
       <c r="C98" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D98" s="10">
         <v>7</v>
@@ -18601,7 +18631,7 @@
         <v>294</v>
       </c>
       <c r="C99" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D99" s="24">
         <v>6</v>
@@ -18765,7 +18795,7 @@
         <v>310</v>
       </c>
       <c r="C100" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D100" s="10">
         <v>5</v>
@@ -18929,7 +18959,7 @@
         <v>312</v>
       </c>
       <c r="C101" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D101" s="24">
         <v>4</v>
@@ -19093,7 +19123,7 @@
         <v>314</v>
       </c>
       <c r="C102" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D102" s="10">
         <v>3</v>
@@ -19257,7 +19287,7 @@
         <v>317</v>
       </c>
       <c r="C103" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D103" s="24">
         <v>2</v>
@@ -19421,7 +19451,7 @@
         <v>319</v>
       </c>
       <c r="C104" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D104" s="10">
         <v>1</v>
@@ -19585,7 +19615,7 @@
         <v>321</v>
       </c>
       <c r="C105" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D105" s="24">
         <v>8</v>
@@ -19749,7 +19779,7 @@
         <v>322</v>
       </c>
       <c r="C106" s="10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D106" s="10">
         <v>7</v>
@@ -19913,7 +19943,7 @@
         <v>112</v>
       </c>
       <c r="C107" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D107" s="24">
         <v>6</v>
@@ -20077,7 +20107,7 @@
         <v>325</v>
       </c>
       <c r="C108" s="10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D108" s="10">
         <v>5</v>
@@ -20241,7 +20271,7 @@
         <v>328</v>
       </c>
       <c r="C109" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D109" s="24">
         <v>4</v>
@@ -20405,7 +20435,7 @@
         <v>330</v>
       </c>
       <c r="C110" s="10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D110" s="10">
         <v>3</v>
@@ -20569,7 +20599,7 @@
         <v>314</v>
       </c>
       <c r="C111" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D111" s="24">
         <v>2</v>
@@ -20733,7 +20763,7 @@
         <v>334</v>
       </c>
       <c r="C112" s="10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D112" s="10">
         <v>1</v>
@@ -20897,7 +20927,7 @@
         <v>337</v>
       </c>
       <c r="C113" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D113" s="24">
         <v>5</v>
@@ -21061,7 +21091,7 @@
         <v>339</v>
       </c>
       <c r="C114" s="10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D114" s="10">
         <v>4</v>
@@ -21225,7 +21255,7 @@
         <v>340</v>
       </c>
       <c r="C115" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D115" s="24">
         <v>3</v>
@@ -21389,7 +21419,7 @@
         <v>342</v>
       </c>
       <c r="C116" s="10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D116" s="10">
         <v>2</v>
@@ -21553,7 +21583,7 @@
         <v>344</v>
       </c>
       <c r="C117" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D117" s="24">
         <v>1</v>
@@ -21717,7 +21747,7 @@
         <v>78</v>
       </c>
       <c r="C118" s="10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D118" s="10">
         <v>6</v>
@@ -21881,7 +21911,7 @@
         <v>348</v>
       </c>
       <c r="C119" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D119" s="24">
         <v>5</v>
@@ -22045,7 +22075,7 @@
         <v>350</v>
       </c>
       <c r="C120" s="10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D120" s="10">
         <v>4</v>
@@ -22209,7 +22239,7 @@
         <v>352</v>
       </c>
       <c r="C121" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D121" s="24">
         <v>3</v>
@@ -22373,7 +22403,7 @@
         <v>355</v>
       </c>
       <c r="C122" s="10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D122" s="10">
         <v>2</v>
@@ -22537,7 +22567,7 @@
         <v>357</v>
       </c>
       <c r="C123" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D123" s="24">
         <v>1</v>
@@ -22701,7 +22731,7 @@
         <v>360</v>
       </c>
       <c r="C124" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D124" s="10">
         <v>6</v>
@@ -22865,7 +22895,7 @@
         <v>363</v>
       </c>
       <c r="C125" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D125" s="24">
         <v>5</v>
@@ -23029,7 +23059,7 @@
         <v>365</v>
       </c>
       <c r="C126" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D126" s="10">
         <v>4</v>
@@ -23193,7 +23223,7 @@
         <v>367</v>
       </c>
       <c r="C127" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D127" s="24">
         <v>3</v>
@@ -23357,7 +23387,7 @@
         <v>369</v>
       </c>
       <c r="C128" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D128" s="10">
         <v>2</v>
@@ -23521,7 +23551,7 @@
         <v>371</v>
       </c>
       <c r="C129" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D129" s="24">
         <v>1</v>
@@ -23685,7 +23715,7 @@
         <v>373</v>
       </c>
       <c r="C130" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D130" s="10">
         <v>3</v>
@@ -23849,7 +23879,7 @@
         <v>375</v>
       </c>
       <c r="C131" s="24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D131" s="24">
         <v>2</v>
@@ -24013,7 +24043,7 @@
         <v>377</v>
       </c>
       <c r="C132" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D132" s="10">
         <v>1</v>
@@ -24177,7 +24207,7 @@
         <v>380</v>
       </c>
       <c r="C133" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" s="24">
         <v>11</v>
@@ -24341,7 +24371,7 @@
         <v>382</v>
       </c>
       <c r="C134" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D134" s="10">
         <v>10</v>
@@ -24505,7 +24535,7 @@
         <v>384</v>
       </c>
       <c r="C135" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D135" s="24">
         <v>9</v>
@@ -24669,7 +24699,7 @@
         <v>386</v>
       </c>
       <c r="C136" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D136" s="10">
         <v>8</v>
@@ -24833,7 +24863,7 @@
         <v>389</v>
       </c>
       <c r="C137" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D137" s="24">
         <v>7</v>
@@ -24997,7 +25027,7 @@
         <v>391</v>
       </c>
       <c r="C138" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D138" s="10">
         <v>6</v>
@@ -25161,7 +25191,7 @@
         <v>394</v>
       </c>
       <c r="C139" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D139" s="24">
         <v>5</v>
@@ -25325,7 +25355,7 @@
         <v>272</v>
       </c>
       <c r="C140" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D140" s="10">
         <v>4</v>
@@ -25489,7 +25519,7 @@
         <v>397</v>
       </c>
       <c r="C141" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D141" s="24">
         <v>3</v>
@@ -25653,7 +25683,7 @@
         <v>398</v>
       </c>
       <c r="C142" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D142" s="10">
         <v>2</v>
@@ -25817,7 +25847,7 @@
         <v>399</v>
       </c>
       <c r="C143" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D143" s="24">
         <v>1</v>
@@ -25981,7 +26011,7 @@
         <v>402</v>
       </c>
       <c r="C144" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D144" s="10">
         <v>5</v>
@@ -26145,7 +26175,7 @@
         <v>363</v>
       </c>
       <c r="C145" s="24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D145" s="24">
         <v>4</v>
@@ -26309,7 +26339,7 @@
         <v>404</v>
       </c>
       <c r="C146" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D146" s="10">
         <v>3</v>
@@ -26473,7 +26503,7 @@
         <v>406</v>
       </c>
       <c r="C147" s="24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D147" s="24">
         <v>2</v>
@@ -26637,7 +26667,7 @@
         <v>408</v>
       </c>
       <c r="C148" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D148" s="10">
         <v>1</v>
@@ -26801,10 +26831,10 @@
         <v>412</v>
       </c>
       <c r="C149" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D149" s="24">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E149" s="24" t="s">
         <v>413</v>
@@ -26965,10 +26995,10 @@
         <v>414</v>
       </c>
       <c r="C150" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D150" s="10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E150" s="10" t="s">
         <v>415</v>
@@ -27129,10 +27159,10 @@
         <v>96</v>
       </c>
       <c r="C151" s="24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D151" s="24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E151" s="24" t="s">
         <v>408</v>
@@ -27283,6 +27313,990 @@
       </c>
       <c r="BB151" s="24" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A152" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B152" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C152" s="10">
+        <v>2</v>
+      </c>
+      <c r="D152" s="10">
+        <v>3</v>
+      </c>
+      <c r="E152" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="F152" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G152" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="H152" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I152" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="J152" s="12">
+        <v>1.92</v>
+      </c>
+      <c r="K152" s="10">
+        <v>11</v>
+      </c>
+      <c r="L152" s="13">
+        <v>12</v>
+      </c>
+      <c r="M152" s="10">
+        <v>12</v>
+      </c>
+      <c r="N152" s="36">
+        <v>20.2</v>
+      </c>
+      <c r="O152" s="14">
+        <v>50</v>
+      </c>
+      <c r="P152" s="14">
+        <v>21.9</v>
+      </c>
+      <c r="Q152" s="15">
+        <v>2.159</v>
+      </c>
+      <c r="R152" s="41">
+        <v>0.66</v>
+      </c>
+      <c r="S152" s="28">
+        <v>6.1</v>
+      </c>
+      <c r="T152" s="17">
+        <v>430</v>
+      </c>
+      <c r="U152" s="17">
+        <v>928</v>
+      </c>
+      <c r="V152" s="10">
+        <v>962</v>
+      </c>
+      <c r="W152" s="10">
+        <v>30</v>
+      </c>
+      <c r="X152" s="10">
+        <v>2</v>
+      </c>
+      <c r="Y152" s="10">
+        <v>8</v>
+      </c>
+      <c r="Z152" s="10">
+        <v>1</v>
+      </c>
+      <c r="AA152" s="10">
+        <v>39</v>
+      </c>
+      <c r="AB152" s="10">
+        <v>7</v>
+      </c>
+      <c r="AC152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE152" s="10">
+        <v>5</v>
+      </c>
+      <c r="AF152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG152" s="10">
+        <v>1</v>
+      </c>
+      <c r="AH152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ152" s="10">
+        <v>27</v>
+      </c>
+      <c r="AK152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL152" s="10">
+        <v>6</v>
+      </c>
+      <c r="AM152" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN152" s="10">
+        <v>1</v>
+      </c>
+      <c r="AO152" s="18">
+        <v>3</v>
+      </c>
+      <c r="AP152" s="47">
+        <v>40</v>
+      </c>
+      <c r="AQ152" s="19">
+        <v>-4</v>
+      </c>
+      <c r="AR152" s="19">
+        <v>-1071</v>
+      </c>
+      <c r="AS152" s="10">
+        <v>4</v>
+      </c>
+      <c r="AT152" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU152" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AV152" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AW152" s="21">
+        <v>-0.2</v>
+      </c>
+      <c r="AX152" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="AY152" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ152" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BA152" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB152" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A153" s="23" t="s">
+        <v>411</v>
+      </c>
+      <c r="B153" s="24" t="s">
+        <v>417</v>
+      </c>
+      <c r="C153" s="24">
+        <v>2</v>
+      </c>
+      <c r="D153" s="24">
+        <v>2</v>
+      </c>
+      <c r="E153" s="24" t="s">
+        <v>418</v>
+      </c>
+      <c r="F153" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="G153" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="H153" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="I153" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J153" s="35">
+        <v>0.63</v>
+      </c>
+      <c r="K153" s="24">
+        <v>2</v>
+      </c>
+      <c r="L153" s="13">
+        <v>8</v>
+      </c>
+      <c r="M153" s="24">
+        <v>3</v>
+      </c>
+      <c r="N153" s="27">
+        <v>14.6</v>
+      </c>
+      <c r="O153" s="27">
+        <v>50</v>
+      </c>
+      <c r="P153" s="27">
+        <v>26.6</v>
+      </c>
+      <c r="Q153" s="15">
+        <v>1.907</v>
+      </c>
+      <c r="R153" s="41">
+        <v>0.62</v>
+      </c>
+      <c r="S153" s="28">
+        <v>5.8</v>
+      </c>
+      <c r="T153" s="29">
+        <v>345</v>
+      </c>
+      <c r="U153" s="29">
+        <v>659</v>
+      </c>
+      <c r="V153" s="24">
+        <v>389</v>
+      </c>
+      <c r="W153" s="24">
+        <v>12</v>
+      </c>
+      <c r="X153" s="24">
+        <v>0</v>
+      </c>
+      <c r="Y153" s="24">
+        <v>5</v>
+      </c>
+      <c r="Z153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AA153" s="24">
+        <v>27</v>
+      </c>
+      <c r="AB153" s="24">
+        <v>4</v>
+      </c>
+      <c r="AC153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AD153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AE153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AF153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG153" s="24">
+        <v>3</v>
+      </c>
+      <c r="AH153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AI153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AJ153" s="24">
+        <v>23</v>
+      </c>
+      <c r="AK153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AL153" s="24">
+        <v>1</v>
+      </c>
+      <c r="AM153" s="24">
+        <v>0</v>
+      </c>
+      <c r="AN153" s="24">
+        <v>3</v>
+      </c>
+      <c r="AO153" s="19">
+        <v>-5</v>
+      </c>
+      <c r="AP153" s="19">
+        <v>-1115</v>
+      </c>
+      <c r="AQ153" s="19">
+        <v>-45</v>
+      </c>
+      <c r="AR153" s="19">
+        <v>-2560</v>
+      </c>
+      <c r="AS153" s="24">
+        <v>5</v>
+      </c>
+      <c r="AT153" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU153" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="AV153" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AW153" s="43">
+        <v>-0.95</v>
+      </c>
+      <c r="AX153" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="AY153" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ153" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="BA153" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="BB153" s="24" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A154" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B154" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="C154" s="10">
+        <v>2</v>
+      </c>
+      <c r="D154" s="10">
+        <v>1</v>
+      </c>
+      <c r="E154" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="F154" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="G154" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H154" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I154" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J154" s="35">
+        <v>0</v>
+      </c>
+      <c r="K154" s="10">
+        <v>0</v>
+      </c>
+      <c r="L154" s="33">
+        <v>0</v>
+      </c>
+      <c r="M154" s="10">
+        <v>0</v>
+      </c>
+      <c r="N154" s="14">
+        <v>0</v>
+      </c>
+      <c r="O154" s="14">
+        <v>0</v>
+      </c>
+      <c r="P154" s="14">
+        <v>100</v>
+      </c>
+      <c r="Q154" s="49">
+        <v>0.58</v>
+      </c>
+      <c r="R154" s="41">
+        <v>0.58</v>
+      </c>
+      <c r="S154" s="28">
+        <v>0</v>
+      </c>
+      <c r="T154" s="17">
+        <v>434</v>
+      </c>
+      <c r="U154" s="17">
+        <v>252</v>
+      </c>
+      <c r="V154" s="10">
+        <v>0</v>
+      </c>
+      <c r="W154" s="10">
+        <v>0</v>
+      </c>
+      <c r="X154" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y154" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AC154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AH154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AK154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN154" s="10">
+        <v>0</v>
+      </c>
+      <c r="AO154" s="47">
+        <v>0</v>
+      </c>
+      <c r="AP154" s="47">
+        <v>-15</v>
+      </c>
+      <c r="AQ154" s="47">
+        <v>0</v>
+      </c>
+      <c r="AR154" s="47">
+        <v>-15</v>
+      </c>
+      <c r="AS154" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="AT154" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU154" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="AV154" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AW154" s="21">
+        <v>-0.8</v>
+      </c>
+      <c r="AX154" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="AY154" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ154" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BA154" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB154" s="10" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="155" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A155" s="23" t="s">
+        <v>420</v>
+      </c>
+      <c r="B155" s="24" t="s">
+        <v>421</v>
+      </c>
+      <c r="C155" s="24">
+        <v>1</v>
+      </c>
+      <c r="D155" s="24">
+        <v>3</v>
+      </c>
+      <c r="E155" s="24" t="s">
+        <v>422</v>
+      </c>
+      <c r="F155" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="G155" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="H155" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="I155" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="J155" s="45">
+        <v>3.5</v>
+      </c>
+      <c r="K155" s="24">
+        <v>5</v>
+      </c>
+      <c r="L155" s="24">
+        <v>4</v>
+      </c>
+      <c r="M155" s="24">
+        <v>9</v>
+      </c>
+      <c r="N155" s="27">
+        <v>6.4</v>
+      </c>
+      <c r="O155" s="27">
+        <v>50</v>
+      </c>
+      <c r="P155" s="27">
+        <v>27.6</v>
+      </c>
+      <c r="Q155" s="15">
+        <v>1.689</v>
+      </c>
+      <c r="R155" s="26">
+        <v>1.12</v>
+      </c>
+      <c r="S155" s="27">
+        <v>8.3</v>
+      </c>
+      <c r="T155" s="29">
+        <v>506</v>
+      </c>
+      <c r="U155" s="29">
+        <v>855</v>
+      </c>
+      <c r="V155" s="24">
+        <v>553</v>
+      </c>
+      <c r="W155" s="24">
+        <v>17</v>
+      </c>
+      <c r="X155" s="24">
+        <v>5</v>
+      </c>
+      <c r="Y155" s="24">
+        <v>2</v>
+      </c>
+      <c r="Z155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AA155" s="24">
+        <v>14</v>
+      </c>
+      <c r="AB155" s="24">
+        <v>7</v>
+      </c>
+      <c r="AC155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AD155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AE155" s="24">
+        <v>1</v>
+      </c>
+      <c r="AF155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG155" s="24">
+        <v>3</v>
+      </c>
+      <c r="AH155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AI155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AJ155" s="24">
+        <v>6</v>
+      </c>
+      <c r="AK155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AL155" s="24">
+        <v>4</v>
+      </c>
+      <c r="AM155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AN155" s="24">
+        <v>0</v>
+      </c>
+      <c r="AO155" s="18">
+        <v>8</v>
+      </c>
+      <c r="AP155" s="18">
+        <v>233</v>
+      </c>
+      <c r="AQ155" s="18">
+        <v>11</v>
+      </c>
+      <c r="AR155" s="18">
+        <v>1179</v>
+      </c>
+      <c r="AS155" s="24">
+        <v>3</v>
+      </c>
+      <c r="AT155" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU155" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="AV155" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="AW155" s="43">
+        <v>0.5</v>
+      </c>
+      <c r="AX155" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="AY155" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ155" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="BA155" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB155" s="24" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="156" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A156" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="B156" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="C156" s="10">
+        <v>1</v>
+      </c>
+      <c r="D156" s="10">
+        <v>2</v>
+      </c>
+      <c r="E156" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="F156" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="G156" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H156" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I156" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J156" s="45">
+        <v>3</v>
+      </c>
+      <c r="K156" s="10">
+        <v>13</v>
+      </c>
+      <c r="L156" s="13">
+        <v>6</v>
+      </c>
+      <c r="M156" s="10">
+        <v>5</v>
+      </c>
+      <c r="N156" s="14">
+        <v>8</v>
+      </c>
+      <c r="O156" s="14">
+        <v>75</v>
+      </c>
+      <c r="P156" s="14">
+        <v>36.9</v>
+      </c>
+      <c r="Q156" s="15">
+        <v>2.453</v>
+      </c>
+      <c r="R156" s="16">
+        <v>1.69</v>
+      </c>
+      <c r="S156" s="14">
+        <v>7.7</v>
+      </c>
+      <c r="T156" s="17">
+        <v>540</v>
+      </c>
+      <c r="U156" s="17">
+        <v>1325</v>
+      </c>
+      <c r="V156" s="10">
+        <v>431</v>
+      </c>
+      <c r="W156" s="10">
+        <v>13</v>
+      </c>
+      <c r="X156" s="10">
+        <v>6</v>
+      </c>
+      <c r="Y156" s="10">
+        <v>2</v>
+      </c>
+      <c r="Z156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA156" s="10">
+        <v>18</v>
+      </c>
+      <c r="AB156" s="10">
+        <v>6</v>
+      </c>
+      <c r="AC156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AG156" s="10">
+        <v>4</v>
+      </c>
+      <c r="AH156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AI156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AJ156" s="10">
+        <v>12</v>
+      </c>
+      <c r="AK156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AL156" s="10">
+        <v>2</v>
+      </c>
+      <c r="AM156" s="10">
+        <v>0</v>
+      </c>
+      <c r="AN156" s="10">
+        <v>1</v>
+      </c>
+      <c r="AO156" s="18">
+        <v>4</v>
+      </c>
+      <c r="AP156" s="18">
+        <v>778</v>
+      </c>
+      <c r="AQ156" s="19">
+        <v>-1</v>
+      </c>
+      <c r="AR156" s="18">
+        <v>1457</v>
+      </c>
+      <c r="AS156" s="10">
+        <v>3</v>
+      </c>
+      <c r="AT156" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU156" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="AV156" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="AW156" s="31">
+        <v>1.65</v>
+      </c>
+      <c r="AX156" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="AY156" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ156" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BA156" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB156" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1" spans="1:54" x14ac:dyDescent="0.25">
+      <c r="A157" s="23" t="s">
+        <v>420</v>
+      </c>
+      <c r="B157" s="24" t="s">
+        <v>424</v>
+      </c>
+      <c r="C157" s="24">
+        <v>1</v>
+      </c>
+      <c r="D157" s="24">
+        <v>1</v>
+      </c>
+      <c r="E157" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="F157" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="G157" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="H157" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="I157" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="J157" s="16">
+        <v>8.67</v>
+      </c>
+      <c r="K157" s="24">
+        <v>15</v>
+      </c>
+      <c r="L157" s="24">
+        <v>3</v>
+      </c>
+      <c r="M157" s="24">
+        <v>11</v>
+      </c>
+      <c r="N157" s="27">
+        <v>4.3</v>
+      </c>
+      <c r="O157" s="27">
+        <v>61.9</v>
+      </c>
+      <c r="P157" s="27">
+        <v>41.1</v>
+      </c>
+      <c r="Q157" s="15">
+        <v>3.534</v>
+      </c>
+      <c r="R157" s="16">
+        <v>3.07</v>
+      </c>
+      <c r="S157" s="46">
+        <v>9.7</v>
+      </c>
+      <c r="T157" s="29">
+        <v>652</v>
+      </c>
+      <c r="U157" s="29">
+        <v>2303</v>
+      </c>
+      <c r="V157" s="24">
+        <v>988</v>
+      </c>
+      <c r="W157" s="24">
+        <v>27</v>
+      </c>
+      <c r="X157" s="24">
+        <v>10</v>
+      </c>
+      <c r="Y157" s="24">
+        <v>6</v>
+      </c>
+      <c r="Z157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AA157" s="24">
+        <v>25</v>
+      </c>
+      <c r="AB157" s="24">
+        <v>2</v>
+      </c>
+      <c r="AC157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AD157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AE157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AF157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AG157" s="24">
+        <v>1</v>
+      </c>
+      <c r="AH157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AI157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AJ157" s="24">
+        <v>22</v>
+      </c>
+      <c r="AK157" s="24">
+        <v>1</v>
+      </c>
+      <c r="AL157" s="24">
+        <v>1</v>
+      </c>
+      <c r="AM157" s="24">
+        <v>0</v>
+      </c>
+      <c r="AN157" s="24">
+        <v>2</v>
+      </c>
+      <c r="AO157" s="18">
+        <v>20</v>
+      </c>
+      <c r="AP157" s="18">
+        <v>868</v>
+      </c>
+      <c r="AQ157" s="18">
+        <v>24</v>
+      </c>
+      <c r="AR157" s="18">
+        <v>1615</v>
+      </c>
+      <c r="AS157" s="24">
+        <v>4</v>
+      </c>
+      <c r="AT157" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AU157" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="AV157" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="AW157" s="31">
+        <v>1.75</v>
+      </c>
+      <c r="AX157" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="AY157" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="AZ157" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="BA157" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="BB157" s="24" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -27311,7 +28325,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="50" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="B1" s="50"/>
       <c r="C1" s="50"/>
@@ -27336,46 +28350,46 @@
         <v>5</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="C2" s="51" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="D2" s="51" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="E2" s="51" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="F2" s="51" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="G2" s="51" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="H2" s="51" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="I2" s="51" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="J2" s="51" t="s">
-        <v>425</v>
+        <v>435</v>
       </c>
       <c r="K2" s="51" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="L2" s="51" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="M2" s="51" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="N2" s="51" t="s">
-        <v>429</v>
+        <v>439</v>
       </c>
       <c r="O2" s="51" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="P2" s="51" t="s">
         <v>81</v>
@@ -27384,7 +28398,7 @@
         <v>59</v>
       </c>
       <c r="R2" s="51" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -27392,22 +28406,22 @@
         <v>87</v>
       </c>
       <c r="B3" s="10">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C3" s="10">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" s="10">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E3" s="53">
-        <v>0.48484848484848486</v>
+        <v>0.4852941176470588</v>
       </c>
       <c r="F3" s="12">
-        <v>2.44</v>
+        <v>2.4</v>
       </c>
       <c r="G3" s="10">
-        <v>9.9</v>
+        <v>9.8</v>
       </c>
       <c r="H3" s="13">
         <v>8.1</v>
@@ -27416,19 +28430,19 @@
         <v>7.2</v>
       </c>
       <c r="J3" s="28">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="K3" s="17">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="L3" s="17">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="M3" s="54">
-        <v>23.9</v>
+        <v>24</v>
       </c>
       <c r="N3" s="54">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="O3" s="10">
         <v>23</v>
@@ -27437,10 +28451,10 @@
         <v>21</v>
       </c>
       <c r="Q3" s="10">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>296</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -27496,7 +28510,7 @@
         <v>17</v>
       </c>
       <c r="R4" s="24" t="s">
-        <v>432</v>
+        <v>443</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -27552,7 +28566,7 @@
         <v>8</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>433</v>
+        <v>444</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -27608,287 +28622,287 @@
         <v>8</v>
       </c>
       <c r="R6" s="24" t="s">
-        <v>434</v>
+        <v>445</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="52" t="s">
-        <v>102</v>
+        <v>148</v>
       </c>
       <c r="B7" s="10">
+        <v>7</v>
+      </c>
+      <c r="C7" s="10">
         <v>6</v>
       </c>
-      <c r="C7" s="10">
-        <v>2</v>
-      </c>
       <c r="D7" s="10">
-        <v>4</v>
-      </c>
-      <c r="E7" s="59">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F7" s="12">
-        <v>2.25</v>
+        <v>1</v>
+      </c>
+      <c r="E7" s="58">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F7" s="16">
+        <v>7.65</v>
       </c>
       <c r="G7" s="10">
-        <v>10.8</v>
-      </c>
-      <c r="H7" s="13">
-        <v>8.3</v>
+        <v>11</v>
+      </c>
+      <c r="H7" s="10">
+        <v>5.4</v>
       </c>
       <c r="I7" s="10">
-        <v>4.8</v>
+        <v>9.9</v>
       </c>
       <c r="J7" s="14">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="K7" s="17">
-        <v>496</v>
+        <v>580</v>
       </c>
       <c r="L7" s="17">
-        <v>1330</v>
+        <v>1244</v>
       </c>
       <c r="M7" s="54">
-        <v>35</v>
+        <v>29.7</v>
       </c>
       <c r="N7" s="54">
-        <v>52.9</v>
+        <v>57.2</v>
       </c>
       <c r="O7" s="10">
-        <v>17.7</v>
+        <v>17</v>
       </c>
       <c r="P7" s="10">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R7" s="10" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="55" t="s">
-        <v>148</v>
+        <v>102</v>
       </c>
       <c r="B8" s="24">
+        <v>7</v>
+      </c>
+      <c r="C8" s="24">
+        <v>2</v>
+      </c>
+      <c r="D8" s="24">
         <v>5</v>
       </c>
-      <c r="C8" s="24">
-        <v>4</v>
-      </c>
-      <c r="D8" s="24">
-        <v>1</v>
-      </c>
-      <c r="E8" s="58">
-        <v>0.8</v>
-      </c>
-      <c r="F8" s="16">
-        <v>8.28</v>
+      <c r="E8" s="59">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F8" s="26">
+        <v>1.93</v>
       </c>
       <c r="G8" s="24">
-        <v>11.4</v>
+        <v>9.3</v>
       </c>
       <c r="H8" s="13">
-        <v>6.2</v>
+        <v>7.1</v>
       </c>
       <c r="I8" s="24">
-        <v>9.8</v>
-      </c>
-      <c r="J8" s="27">
-        <v>7.7</v>
+        <v>4.1</v>
+      </c>
+      <c r="J8" s="28">
+        <v>6.5</v>
       </c>
       <c r="K8" s="29">
-        <v>580</v>
+        <v>487</v>
       </c>
       <c r="L8" s="29">
-        <v>1110</v>
+        <v>1176</v>
       </c>
       <c r="M8" s="57">
-        <v>27.9</v>
+        <v>44.3</v>
       </c>
       <c r="N8" s="57">
-        <v>57.7</v>
+        <v>45.3</v>
       </c>
       <c r="O8" s="24">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="P8" s="24">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="24">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R8" s="24" t="s">
-        <v>436</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B9" s="10">
         <v>4</v>
       </c>
       <c r="C9" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="10">
-        <v>2</v>
-      </c>
-      <c r="E9" s="53">
-        <v>0.5</v>
-      </c>
-      <c r="F9" s="16">
-        <v>4.37</v>
+        <v>3</v>
+      </c>
+      <c r="E9" s="59">
+        <v>0.25</v>
+      </c>
+      <c r="F9" s="12">
+        <v>2.27</v>
       </c>
       <c r="G9" s="10">
-        <v>11.5</v>
+        <v>7.8</v>
       </c>
       <c r="H9" s="13">
-        <v>7.8</v>
+        <v>7.3</v>
       </c>
       <c r="I9" s="10">
+        <v>9.5</v>
+      </c>
+      <c r="J9" s="28">
+        <v>5.9</v>
+      </c>
+      <c r="K9" s="17">
+        <v>450</v>
+      </c>
+      <c r="L9" s="17">
+        <v>937</v>
+      </c>
+      <c r="M9" s="54">
+        <v>26.3</v>
+      </c>
+      <c r="N9" s="54">
+        <v>57.2</v>
+      </c>
+      <c r="O9" s="10">
+        <v>39.5</v>
+      </c>
+      <c r="P9" s="10">
         <v>3</v>
       </c>
-      <c r="J9" s="14">
-        <v>8.8</v>
-      </c>
-      <c r="K9" s="17">
-        <v>558</v>
-      </c>
-      <c r="L9" s="17">
-        <v>1031</v>
-      </c>
-      <c r="M9" s="54">
-        <v>30.4</v>
-      </c>
-      <c r="N9" s="54">
-        <v>51.4</v>
-      </c>
-      <c r="O9" s="10">
-        <v>17.3</v>
-      </c>
-      <c r="P9" s="10">
-        <v>1</v>
-      </c>
       <c r="Q9" s="10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>329</v>
+        <v>448</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="55" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="B10" s="24">
+        <v>4</v>
+      </c>
+      <c r="C10" s="24">
+        <v>2</v>
+      </c>
+      <c r="D10" s="24">
+        <v>2</v>
+      </c>
+      <c r="E10" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="F10" s="16">
+        <v>4.37</v>
+      </c>
+      <c r="G10" s="24">
+        <v>11.5</v>
+      </c>
+      <c r="H10" s="13">
+        <v>7.8</v>
+      </c>
+      <c r="I10" s="24">
         <v>3</v>
       </c>
-      <c r="C10" s="24">
+      <c r="J10" s="27">
+        <v>8.8</v>
+      </c>
+      <c r="K10" s="29">
+        <v>558</v>
+      </c>
+      <c r="L10" s="29">
+        <v>1031</v>
+      </c>
+      <c r="M10" s="57">
+        <v>30.4</v>
+      </c>
+      <c r="N10" s="57">
+        <v>51.4</v>
+      </c>
+      <c r="O10" s="24">
+        <v>17.3</v>
+      </c>
+      <c r="P10" s="24">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="24">
         <v>3</v>
       </c>
-      <c r="D10" s="24">
-        <v>0</v>
-      </c>
-      <c r="E10" s="58">
-        <v>1</v>
-      </c>
-      <c r="F10" s="45">
-        <v>3.92</v>
-      </c>
-      <c r="G10" s="24">
-        <v>6</v>
-      </c>
-      <c r="H10" s="24">
-        <v>5</v>
-      </c>
-      <c r="I10" s="24">
-        <v>9.3</v>
-      </c>
-      <c r="J10" s="28">
-        <v>1.1</v>
-      </c>
-      <c r="K10" s="29">
-        <v>358</v>
-      </c>
-      <c r="L10" s="29">
-        <v>767</v>
-      </c>
-      <c r="M10" s="57">
-        <v>18.6</v>
-      </c>
-      <c r="N10" s="57">
-        <v>42.1</v>
-      </c>
-      <c r="O10" s="24">
-        <v>49.3</v>
-      </c>
-      <c r="P10" s="24">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="24">
-        <v>0</v>
-      </c>
       <c r="R10" s="24" t="s">
-        <v>437</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="52" t="s">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="B11" s="10">
         <v>3</v>
       </c>
       <c r="C11" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D11" s="10">
-        <v>2</v>
-      </c>
-      <c r="E11" s="59">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="F11" s="12">
-        <v>2.02</v>
+        <v>0</v>
+      </c>
+      <c r="E11" s="58">
+        <v>1</v>
+      </c>
+      <c r="F11" s="45">
+        <v>3.92</v>
       </c>
       <c r="G11" s="10">
         <v>6</v>
       </c>
-      <c r="H11" s="13">
-        <v>7.7</v>
+      <c r="H11" s="10">
+        <v>5</v>
       </c>
       <c r="I11" s="10">
-        <v>11</v>
+        <v>9.3</v>
       </c>
       <c r="J11" s="28">
-        <v>5.2</v>
+        <v>1.1</v>
       </c>
       <c r="K11" s="17">
-        <v>419</v>
+        <v>358</v>
       </c>
       <c r="L11" s="17">
-        <v>807</v>
+        <v>767</v>
       </c>
       <c r="M11" s="54">
-        <v>22.7</v>
+        <v>18.6</v>
       </c>
       <c r="N11" s="54">
-        <v>51.2</v>
+        <v>42.1</v>
       </c>
       <c r="O11" s="10">
-        <v>48.3</v>
+        <v>49.3</v>
       </c>
       <c r="P11" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q11" s="10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" s="10" t="s">
-        <v>438</v>
+        <v>449</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -28920,7 +29934,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
-        <v>439</v>
+        <v>450</v>
       </c>
       <c r="B1" s="60"/>
       <c r="C1" s="60"/>
@@ -28930,59 +29944,59 @@
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="61" t="s">
-        <v>440</v>
+        <v>451</v>
       </c>
       <c r="B2" s="61" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="C2" s="61" t="s">
-        <v>442</v>
+        <v>453</v>
       </c>
       <c r="D2" s="61" t="s">
-        <v>443</v>
+        <v>454</v>
       </c>
       <c r="E2" s="61" t="s">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="F2" s="61" t="s">
-        <v>445</v>
+        <v>456</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="52" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="B3" s="10">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C3" s="10">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D3" s="10">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E3" s="10">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F3" s="10">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="55" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="B4" s="24">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D4" s="24">
         <v>35</v>
       </c>
       <c r="E4" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4" s="24">
         <v>42</v>
@@ -28990,90 +30004,90 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="52" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="B5" s="10">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" s="10">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D5" s="10">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5" s="10">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="10">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="55" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="B6" s="56">
-        <v>45.5</v>
+        <v>46.6</v>
       </c>
       <c r="C6" s="56">
-        <v>52.6</v>
+        <v>52</v>
       </c>
       <c r="D6" s="56">
-        <v>53</v>
+        <v>52.2</v>
       </c>
       <c r="E6" s="56">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="F6" s="58">
-        <v>56.8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="52" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="B7" s="45">
-        <v>3.77</v>
+        <v>3.83</v>
       </c>
       <c r="C7" s="45">
-        <v>3.19</v>
+        <v>3.12</v>
       </c>
       <c r="D7" s="45">
-        <v>3.55</v>
+        <v>3.51</v>
       </c>
       <c r="E7" s="12">
-        <v>2.36</v>
+        <v>2.27</v>
       </c>
       <c r="F7" s="16">
-        <v>4.12</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="55" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="B8" s="24">
         <v>10.6</v>
       </c>
       <c r="C8" s="24">
-        <v>10.9</v>
+        <v>10.7</v>
       </c>
       <c r="D8" s="24">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="E8" s="24">
-        <v>9</v>
+        <v>8.8</v>
       </c>
       <c r="F8" s="24">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="B9" s="10">
-        <v>8.7</v>
+        <v>8.5</v>
       </c>
       <c r="C9" s="10">
         <v>7.5</v>
@@ -29082,7 +30096,7 @@
         <v>7.4</v>
       </c>
       <c r="E9" s="10">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="F9" s="10">
         <v>7</v>
@@ -29090,19 +30104,19 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="55" t="s">
-        <v>449</v>
+        <v>460</v>
       </c>
       <c r="B10" s="24">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="C10" s="24">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="D10" s="24">
         <v>5.9</v>
       </c>
       <c r="E10" s="24">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="F10" s="24">
         <v>5.7</v>
@@ -29110,19 +30124,19 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="52" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="B11" s="10">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="C11" s="10">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="D11" s="10">
         <v>7.3</v>
       </c>
       <c r="E11" s="10">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="F11" s="10">
         <v>7.3</v>
@@ -29130,139 +30144,139 @@
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
       <c r="B12" s="24">
-        <v>1018</v>
+        <v>1043</v>
       </c>
       <c r="C12" s="24">
-        <v>1108</v>
+        <v>1092</v>
       </c>
       <c r="D12" s="24">
-        <v>1161</v>
+        <v>1153</v>
       </c>
       <c r="E12" s="24">
-        <v>987</v>
+        <v>961</v>
       </c>
       <c r="F12" s="24">
-        <v>1181</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="52" t="s">
-        <v>452</v>
+        <v>463</v>
       </c>
       <c r="B13" s="10">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="C13" s="10">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D13" s="10">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="E13" s="10">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="F13" s="10">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="55" t="s">
-        <v>453</v>
+        <v>464</v>
       </c>
       <c r="B14" s="24">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
       <c r="C14" s="24">
-        <v>29.1</v>
+        <v>29.8</v>
       </c>
       <c r="D14" s="24">
-        <v>30.9</v>
+        <v>30.8</v>
       </c>
       <c r="E14" s="24">
-        <v>25.2</v>
+        <v>27.5</v>
       </c>
       <c r="F14" s="24">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="52" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="B15" s="10">
-        <v>51</v>
+        <v>51.6</v>
       </c>
       <c r="C15" s="10">
-        <v>56.1</v>
+        <v>55.4</v>
       </c>
       <c r="D15" s="10">
-        <v>57.4</v>
+        <v>57.3</v>
       </c>
       <c r="E15" s="10">
-        <v>53.2</v>
+        <v>51.3</v>
       </c>
       <c r="F15" s="10">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
       <c r="B16" s="24">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="C16" s="24">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="D16" s="24">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="E16" s="24">
-        <v>20.4</v>
+        <v>20.1</v>
       </c>
       <c r="F16" s="24">
-        <v>20</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
       <c r="B17" s="10">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C17" s="10">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="D17" s="10">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="E17" s="10">
-        <v>680</v>
+        <v>667</v>
       </c>
       <c r="F17" s="10">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="55" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="B18" s="24">
-        <v>13.6</v>
+        <v>13.3</v>
       </c>
       <c r="C18" s="24">
         <v>12.3</v>
       </c>
       <c r="D18" s="24">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="E18" s="24">
-        <v>13.8</v>
+        <v>13.6</v>
       </c>
       <c r="F18" s="24">
         <v>11</v>
@@ -29270,7 +30284,7 @@
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="52" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
       <c r="B19" s="10">
         <v>19</v>
@@ -29282,7 +30296,7 @@
         <v>23</v>
       </c>
       <c r="E19" s="10">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F19" s="10">
         <v>23</v>
@@ -29290,7 +30304,7 @@
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="55" t="s">
-        <v>459</v>
+        <v>470</v>
       </c>
       <c r="B20" s="24">
         <v>5</v>
@@ -29330,7 +30344,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
-        <v>460</v>
+        <v>471</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -29342,15 +30356,15 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="B2" s="10">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="64" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="B3" s="56">
         <v>0.5</v>
@@ -29358,39 +30372,39 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="64" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="63" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="64" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="B7" s="24">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="63" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="B8" s="10">
         <v>499</v>
@@ -29398,31 +30412,31 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="64" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="62" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="B13" s="62"/>
       <c r="C13" s="62"/>
@@ -29434,15 +30448,15 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="63" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="64" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
       <c r="B15" s="56">
         <v>0.4</v>
@@ -29450,7 +30464,7 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="63" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="B16" s="53">
         <v>0.5</v>
@@ -29458,31 +30472,31 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="64" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="63" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="63" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="B20" s="10">
         <v>1241</v>
@@ -29490,7 +30504,7 @@
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="62" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
       <c r="B22" s="62"/>
       <c r="C22" s="62"/>
@@ -29502,137 +30516,137 @@
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="65" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="B23" s="65" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="C23" s="65" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="D23" s="65" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="E23" s="65" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="F23" s="65" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="G23" s="65" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="H23" s="65" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="52" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="B24" s="10">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C24" s="58">
-        <v>0.5833333333333334</v>
+        <v>0.56</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="55" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="B25" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" s="58">
-        <v>0.7727272727272727</v>
+        <v>0.6956521739130435</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>495</v>
+        <v>512</v>
       </c>
       <c r="F25" s="33" t="s">
-        <v>501</v>
+        <v>513</v>
       </c>
       <c r="G25" s="24" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="H25" s="24" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="52" t="s">
-        <v>504</v>
+        <v>516</v>
       </c>
       <c r="B26" s="10">
-        <v>22</v>
-      </c>
-      <c r="C26" s="53">
-        <v>0.5454545454545454</v>
+        <v>23</v>
+      </c>
+      <c r="C26" s="58">
+        <v>0.5652173913043478</v>
       </c>
       <c r="D26" s="33" t="s">
-        <v>505</v>
+        <v>517</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>506</v>
+        <v>518</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>507</v>
+        <v>519</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="55" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="B27" s="24">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C27" s="59">
-        <v>0.3902439024390244</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="D27" s="66" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="F27" s="24" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="G27" s="24" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="H27" s="24" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="67" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="B28" s="67"/>
       <c r="C28" s="67"/>
@@ -29644,7 +30658,7 @@
     </row>
     <row r="30" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="62" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="B30" s="62"/>
       <c r="C30" s="62"/>
@@ -29656,19 +30670,19 @@
     </row>
     <row r="31" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="65" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="B31" s="65" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="C31" s="65" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="D31" s="65" t="s">
         <v>9</v>
       </c>
       <c r="E31" s="65" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="F31" s="65" t="s">
         <v>20</v>
@@ -29677,12 +30691,12 @@
         <v>27</v>
       </c>
       <c r="H31" s="65" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="52" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="B32" s="10">
         <v>5</v>
@@ -29691,10 +30705,10 @@
         <v>0.6</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="F32" s="10">
         <v>972</v>
@@ -29703,12 +30717,12 @@
         <v>5</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="55" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="B33" s="24">
         <v>0</v>
@@ -29729,12 +30743,12 @@
         <v>75</v>
       </c>
       <c r="H33" s="24" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="52" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="B34" s="10">
         <v>19</v>
@@ -29743,10 +30757,10 @@
         <v>0.7368421052631579</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="F34" s="10">
         <v>1240</v>
@@ -29755,24 +30769,24 @@
         <v>6</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="55" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="B35" s="24">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C35" s="56">
-        <v>0.4603174603174603</v>
+        <v>0.4621212121212121</v>
       </c>
       <c r="D35" s="24" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="E35" s="24" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="F35" s="24">
         <v>1054</v>
@@ -29781,12 +30795,12 @@
         <v>6</v>
       </c>
       <c r="H35" s="24" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="62" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="B37" s="62"/>
       <c r="C37" s="62"/>
@@ -29798,19 +30812,19 @@
     </row>
     <row r="38" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="65" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="B38" s="65" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="C38" s="65" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="D38" s="65" t="s">
         <v>9</v>
       </c>
       <c r="E38" s="65" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="F38" s="65" t="s">
         <v>20</v>
@@ -29819,64 +30833,64 @@
         <v>27</v>
       </c>
       <c r="H38" s="65" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="52" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="B39" s="10">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C39" s="58">
-        <v>0.56</v>
+        <v>0.5512820512820513</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="F39" s="10">
-        <v>1135</v>
+        <v>1119</v>
       </c>
       <c r="G39" s="10">
         <v>6</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="55" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="B40" s="24">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C40" s="59">
-        <v>0.43243243243243246</v>
+        <v>0.44155844155844154</v>
       </c>
       <c r="D40" s="24" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="E40" s="24" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="F40" s="24">
-        <v>1021</v>
+        <v>1013</v>
       </c>
       <c r="G40" s="24">
         <v>6</v>
       </c>
       <c r="H40" s="24" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="62" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="B42" s="62"/>
       <c r="C42" s="62"/>
@@ -29888,7 +30902,7 @@
     </row>
     <row r="43" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="65" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="B43" s="65" t="s">
         <v>26</v>
@@ -29914,7 +30928,7 @@
     </row>
     <row r="44" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="52" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="B44" s="10">
         <v>24</v>
@@ -29940,10 +30954,10 @@
     </row>
     <row r="45" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="55" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="B45" s="24">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C45" s="24">
         <v>6</v>
@@ -29966,7 +30980,7 @@
     </row>
     <row r="46" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="52" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="B46" s="10">
         <v>24</v>
@@ -29992,7 +31006,7 @@
     </row>
     <row r="47" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="55" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="B47" s="24">
         <v>21</v>
@@ -30013,12 +31027,12 @@
         <v>0</v>
       </c>
       <c r="H47" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="62" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="B49" s="62"/>
       <c r="C49" s="62"/>
@@ -30030,137 +31044,137 @@
     </row>
     <row r="50" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="65" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="B50" s="65" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="C50" s="65" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="D50" s="65" t="s">
         <v>9</v>
       </c>
       <c r="E50" s="65" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="F50" s="65" t="s">
         <v>20</v>
       </c>
       <c r="G50" s="65" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H50" s="65" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="52" t="s">
+        <v>561</v>
+      </c>
+      <c r="B51" s="10">
+        <v>48</v>
+      </c>
+      <c r="C51" s="58">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>562</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="F51" s="10">
+        <v>1010</v>
+      </c>
+      <c r="G51" s="10" t="s">
         <v>550</v>
       </c>
-      <c r="B51" s="10">
-        <v>46</v>
-      </c>
-      <c r="C51" s="58">
-        <v>0.5869565217391305</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>551</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>552</v>
-      </c>
-      <c r="F51" s="10">
-        <v>1030</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>539</v>
-      </c>
       <c r="H51" s="10" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="55" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
       <c r="B52" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C52" s="56">
-        <v>0.46296296296296297</v>
+        <v>0.4642857142857143</v>
       </c>
       <c r="D52" s="24" t="s">
-        <v>555</v>
+        <v>542</v>
       </c>
       <c r="E52" s="24" t="s">
-        <v>556</v>
+        <v>566</v>
       </c>
       <c r="F52" s="24">
         <v>1113</v>
       </c>
       <c r="G52" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H52" s="24" t="s">
-        <v>557</v>
+        <v>567</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="52" t="s">
-        <v>558</v>
+        <v>568</v>
       </c>
       <c r="B53" s="10">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C53" s="58">
-        <v>0.5806451612903226</v>
+        <v>0.59375</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>559</v>
+        <v>569</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="F53" s="10">
-        <v>1205</v>
+        <v>1240</v>
       </c>
       <c r="G53" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="55" t="s">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="B54" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C54" s="59">
-        <v>0.2631578947368421</v>
+        <v>0.25</v>
       </c>
       <c r="D54" s="24" t="s">
-        <v>562</v>
+        <v>572</v>
       </c>
       <c r="E54" s="24" t="s">
-        <v>563</v>
+        <v>573</v>
       </c>
       <c r="F54" s="24">
-        <v>862</v>
+        <v>852</v>
       </c>
       <c r="G54" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H54" s="24" t="s">
-        <v>564</v>
+        <v>574</v>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="62" t="s">
-        <v>565</v>
+        <v>575</v>
       </c>
       <c r="B56" s="62"/>
       <c r="C56" s="62"/>
@@ -30172,10 +31186,10 @@
     </row>
     <row r="57" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="65" t="s">
-        <v>566</v>
+        <v>576</v>
       </c>
       <c r="B57" s="65" t="s">
-        <v>567</v>
+        <v>577</v>
       </c>
       <c r="C57" s="65" t="s">
         <v>5</v>
@@ -30190,15 +31204,15 @@
         <v>6</v>
       </c>
       <c r="G57" s="65" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H57" s="65" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="63" t="s">
-        <v>568</v>
+        <v>578</v>
       </c>
       <c r="B58" s="68">
         <v>31</v>
@@ -30216,15 +31230,15 @@
         <v>58</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H58" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="64" t="s">
-        <v>569</v>
+        <v>579</v>
       </c>
       <c r="B59" s="69">
         <v>2536</v>
@@ -30242,15 +31256,15 @@
         <v>58</v>
       </c>
       <c r="G59" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H59" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="63" t="s">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="B60" s="70">
         <v>11.2</v>
@@ -30268,15 +31282,15 @@
         <v>58</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H60" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="64" t="s">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="B61" s="69">
         <v>756</v>
@@ -30294,15 +31308,15 @@
         <v>58</v>
       </c>
       <c r="G61" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H61" s="24" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="63" t="s">
-        <v>572</v>
+        <v>582</v>
       </c>
       <c r="B62" s="71">
         <v>116</v>
@@ -30320,10 +31334,10 @@
         <v>162</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="H62" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>